<commit_message>
style: ubah tema ke warna cerah ramah warga (Emerald Green & Gold) dan konsep Pemilihan Kepala Desa Karang Satria
</commit_message>
<xml_diff>
--- a/Template_DPS_DPT_Karang_Satria.xlsx
+++ b/Template_DPS_DPT_Karang_Satria.xlsx
@@ -28,13 +28,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FEF08A"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00091F42"/>
+      <color rgb="00064E3B"/>
       <sz val="10"/>
     </font>
     <font>
@@ -51,8 +51,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00091F42"/>
-        <bgColor rgb="00091F42"/>
+        <fgColor rgb="00047857"/>
+        <bgColor rgb="00047857"/>
       </patternFill>
     </fill>
     <fill>
@@ -63,8 +63,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
-        <bgColor rgb="00F8FAFC"/>
+        <fgColor rgb="00F0FDF4"/>
+        <bgColor rgb="00F0FDF4"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,16 +78,16 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="00D4AF37"/>
+        <color rgb="00064E3B"/>
       </left>
       <right style="medium">
-        <color rgb="00D4AF37"/>
+        <color rgb="00064E3B"/>
       </right>
       <top style="medium">
-        <color rgb="00D4AF37"/>
+        <color rgb="00064E3B"/>
       </top>
       <bottom style="medium">
-        <color rgb="00D4AF37"/>
+        <color rgb="00064E3B"/>
       </bottom>
     </border>
     <border>

</xml_diff>